<commit_message>
columns are tken directly from configured matchrules
</commit_message>
<xml_diff>
--- a/backend/data/Customer/People_Soft9.1/PS93_Customer.xlsx
+++ b/backend/data/Customer/People_Soft9.1/PS93_Customer.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PB396RE\Downloads\fuzzy-deduplication - Copy (2)\backend\data\Customer\People_Soft9.1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://people.ey.com/personal/nitish_t_gds_ey_com/Documents/Desktop/DataHEC/backend/data/Customer/People_Soft9.1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1731F96-D715-4464-86F6-9B80B1198C6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{A1731F96-D715-4464-86F6-9B80B1198C6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1CAD9008-F1EA-48FD-A5C4-E32764C8586A}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1255,6 +1255,8 @@
   <dimension ref="A1:O30"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="3" max="3" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.81640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="14.08984375" customWidth="1"/>
     <col min="12" max="12" width="14.1796875" customWidth="1"/>
     <col min="15" max="15" width="18.7265625" customWidth="1"/>

</xml_diff>

<commit_message>
Updated code of header mapping
</commit_message>
<xml_diff>
--- a/backend/data/Customer/People_Soft9.1/PS93_Customer.xlsx
+++ b/backend/data/Customer/People_Soft9.1/PS93_Customer.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://people.ey.com/personal/nitish_t_gds_ey_com/Documents/Desktop/DataHEC/backend/data/Customer/People_Soft9.1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AD739BB\Downloads\DataHEC\backend\data\Customer\People_Soft9.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{A1731F96-D715-4464-86F6-9B80B1198C6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1CAD9008-F1EA-48FD-A5C4-E32764C8586A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{122374BE-CFA9-44D9-BF5D-8962573ECE2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="294">
   <si>
     <t>Cust_Id</t>
   </si>
@@ -37,9 +37,6 @@
     <t>Benton, John B Jr</t>
   </si>
   <si>
-    <t>6649 N Blue Gum St</t>
-  </si>
-  <si>
     <t>New Orleans</t>
   </si>
   <si>
@@ -890,6 +887,21 @@
   </si>
   <si>
     <t>Transaction_Date</t>
+  </si>
+  <si>
+    <t>6649 N Blue Gum St1</t>
+  </si>
+  <si>
+    <t>6649 N Blue Gum St12B</t>
+  </si>
+  <si>
+    <t>3273 State Vt</t>
+  </si>
+  <si>
+    <t>3273 State Rt</t>
+  </si>
+  <si>
+    <t>3274 State Qt</t>
   </si>
 </sst>
 </file>
@@ -1256,7 +1268,8 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.7265625" customWidth="1"/>
+    <col min="10" max="10" width="14.26953125" customWidth="1"/>
     <col min="11" max="11" width="14.08984375" customWidth="1"/>
     <col min="12" max="12" width="14.1796875" customWidth="1"/>
     <col min="15" max="15" width="18.7265625" customWidth="1"/>
@@ -1270,43 +1283,43 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>278</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>288</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.35">
@@ -1314,7 +1327,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C2" t="s">
         <v>2</v>
@@ -1326,34 +1339,34 @@
         <v>4</v>
       </c>
       <c r="F2" t="s">
+        <v>289</v>
+      </c>
+      <c r="G2" t="s">
         <v>5</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>6</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>7</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2">
+        <v>70611</v>
+      </c>
+      <c r="K2" t="s">
         <v>8</v>
       </c>
-      <c r="J2">
-        <v>70116</v>
-      </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>9</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>10</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>11</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>12</v>
-      </c>
-      <c r="O2" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.35">
@@ -1361,46 +1374,46 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" t="s">
         <v>14</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>15</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
+        <v>290</v>
+      </c>
+      <c r="G3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" t="s">
         <v>16</v>
       </c>
-      <c r="F3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>17</v>
-      </c>
-      <c r="I3" t="s">
-        <v>18</v>
       </c>
       <c r="J3">
         <v>70611</v>
       </c>
       <c r="K3" t="s">
+        <v>8</v>
+      </c>
+      <c r="L3" t="s">
         <v>9</v>
       </c>
-      <c r="L3" t="s">
-        <v>10</v>
-      </c>
       <c r="M3" t="s">
+        <v>18</v>
+      </c>
+      <c r="N3" t="s">
         <v>19</v>
       </c>
-      <c r="N3" t="s">
+      <c r="O3" t="s">
         <v>20</v>
-      </c>
-      <c r="O3" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.35">
@@ -1408,46 +1421,46 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" t="s">
         <v>22</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>23</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>24</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>25</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>26</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>27</v>
-      </c>
-      <c r="I4" t="s">
-        <v>28</v>
       </c>
       <c r="J4">
         <v>8014</v>
       </c>
       <c r="K4" t="s">
+        <v>28</v>
+      </c>
+      <c r="L4" t="s">
         <v>29</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>30</v>
       </c>
-      <c r="M4" t="s">
+      <c r="N4" t="s">
         <v>31</v>
       </c>
-      <c r="N4" t="s">
+      <c r="O4" t="s">
         <v>32</v>
-      </c>
-      <c r="O4" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.35">
@@ -1455,46 +1468,46 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" t="s">
         <v>34</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>35</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>36</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>37</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
+        <v>37</v>
+      </c>
+      <c r="I5" t="s">
         <v>38</v>
-      </c>
-      <c r="H5" t="s">
-        <v>38</v>
-      </c>
-      <c r="I5" t="s">
-        <v>39</v>
       </c>
       <c r="J5">
         <v>99501</v>
       </c>
       <c r="K5" t="s">
+        <v>39</v>
+      </c>
+      <c r="L5" t="s">
         <v>40</v>
       </c>
-      <c r="L5" t="s">
+      <c r="M5" t="s">
         <v>41</v>
       </c>
-      <c r="M5" t="s">
+      <c r="N5" t="s">
         <v>42</v>
       </c>
-      <c r="N5" t="s">
+      <c r="O5" t="s">
         <v>43</v>
-      </c>
-      <c r="O5" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.35">
@@ -1502,46 +1515,46 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" t="s">
         <v>45</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>46</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>47</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>48</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>49</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>50</v>
-      </c>
-      <c r="I6" t="s">
-        <v>51</v>
       </c>
       <c r="J6">
         <v>45011</v>
       </c>
       <c r="K6" t="s">
+        <v>51</v>
+      </c>
+      <c r="L6" t="s">
         <v>52</v>
       </c>
-      <c r="L6" t="s">
+      <c r="M6" t="s">
         <v>53</v>
       </c>
-      <c r="M6" t="s">
+      <c r="N6" t="s">
         <v>54</v>
       </c>
-      <c r="N6" t="s">
+      <c r="O6" t="s">
         <v>55</v>
-      </c>
-      <c r="O6" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.35">
@@ -1549,46 +1562,46 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C7" t="s">
+        <v>56</v>
+      </c>
+      <c r="D7" t="s">
         <v>57</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>58</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>59</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>60</v>
       </c>
-      <c r="G7" t="s">
-        <v>61</v>
-      </c>
       <c r="H7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="J7">
         <v>44805</v>
       </c>
       <c r="K7" t="s">
+        <v>61</v>
+      </c>
+      <c r="L7" t="s">
         <v>62</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>63</v>
       </c>
-      <c r="M7" t="s">
+      <c r="N7" t="s">
         <v>64</v>
       </c>
-      <c r="N7" t="s">
+      <c r="O7" t="s">
         <v>65</v>
-      </c>
-      <c r="O7" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.35">
@@ -1596,46 +1609,46 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C8" t="s">
+        <v>66</v>
+      </c>
+      <c r="D8" t="s">
         <v>67</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>68</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>69</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>70</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>71</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>72</v>
-      </c>
-      <c r="I8" t="s">
-        <v>73</v>
       </c>
       <c r="J8">
         <v>60632</v>
       </c>
       <c r="K8" t="s">
+        <v>73</v>
+      </c>
+      <c r="L8" t="s">
         <v>74</v>
       </c>
-      <c r="L8" t="s">
+      <c r="M8" t="s">
         <v>75</v>
       </c>
-      <c r="M8" t="s">
+      <c r="N8" t="s">
         <v>76</v>
       </c>
-      <c r="N8" t="s">
+      <c r="O8" t="s">
         <v>77</v>
-      </c>
-      <c r="O8" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.35">
@@ -1643,46 +1656,46 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C9" t="s">
+        <v>78</v>
+      </c>
+      <c r="D9" t="s">
         <v>79</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>80</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>81</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>82</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>83</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>84</v>
-      </c>
-      <c r="I9" t="s">
-        <v>85</v>
       </c>
       <c r="J9">
         <v>95111</v>
       </c>
       <c r="K9" t="s">
+        <v>85</v>
+      </c>
+      <c r="L9" t="s">
         <v>86</v>
       </c>
-      <c r="L9" t="s">
+      <c r="M9" t="s">
         <v>87</v>
       </c>
-      <c r="M9" t="s">
+      <c r="N9" t="s">
         <v>88</v>
       </c>
-      <c r="N9" t="s">
+      <c r="O9" t="s">
         <v>89</v>
-      </c>
-      <c r="O9" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.35">
@@ -1690,46 +1703,46 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C10" t="s">
+        <v>90</v>
+      </c>
+      <c r="D10" t="s">
         <v>91</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>92</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
+        <v>81</v>
+      </c>
+      <c r="G10" t="s">
         <v>93</v>
       </c>
-      <c r="F10" t="s">
-        <v>82</v>
-      </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>94</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>95</v>
-      </c>
-      <c r="I10" t="s">
-        <v>96</v>
       </c>
       <c r="J10">
         <v>95111</v>
       </c>
       <c r="K10" t="s">
+        <v>85</v>
+      </c>
+      <c r="L10" t="s">
         <v>86</v>
       </c>
-      <c r="L10" t="s">
-        <v>87</v>
-      </c>
       <c r="M10" t="s">
+        <v>96</v>
+      </c>
+      <c r="N10" t="s">
         <v>97</v>
       </c>
-      <c r="N10" t="s">
-        <v>98</v>
-      </c>
       <c r="O10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.35">
@@ -1737,46 +1750,46 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C11" t="s">
+        <v>98</v>
+      </c>
+      <c r="D11" t="s">
         <v>99</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>100</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>101</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>102</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>103</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>104</v>
-      </c>
-      <c r="I11" t="s">
-        <v>105</v>
       </c>
       <c r="J11">
         <v>21224</v>
       </c>
       <c r="K11" t="s">
+        <v>105</v>
+      </c>
+      <c r="L11" t="s">
         <v>106</v>
       </c>
-      <c r="L11" t="s">
+      <c r="M11" t="s">
         <v>107</v>
       </c>
-      <c r="M11" t="s">
+      <c r="N11" t="s">
         <v>108</v>
       </c>
-      <c r="N11" t="s">
+      <c r="O11" t="s">
         <v>109</v>
-      </c>
-      <c r="O11" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.35">
@@ -1784,46 +1797,46 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C12" t="s">
+        <v>110</v>
+      </c>
+      <c r="D12" t="s">
         <v>111</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>112</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
+        <v>101</v>
+      </c>
+      <c r="G12" t="s">
+        <v>102</v>
+      </c>
+      <c r="H12" t="s">
         <v>113</v>
       </c>
-      <c r="F12" t="s">
-        <v>102</v>
-      </c>
-      <c r="G12" t="s">
-        <v>103</v>
-      </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
         <v>114</v>
-      </c>
-      <c r="I12" t="s">
-        <v>115</v>
       </c>
       <c r="J12">
         <v>21224</v>
       </c>
       <c r="K12" t="s">
+        <v>105</v>
+      </c>
+      <c r="L12" t="s">
         <v>106</v>
       </c>
-      <c r="L12" t="s">
-        <v>107</v>
-      </c>
       <c r="M12" t="s">
+        <v>115</v>
+      </c>
+      <c r="N12" t="s">
         <v>116</v>
       </c>
-      <c r="N12" t="s">
+      <c r="O12" t="s">
         <v>117</v>
-      </c>
-      <c r="O12" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.35">
@@ -1831,46 +1844,46 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C13" t="s">
+        <v>118</v>
+      </c>
+      <c r="D13" t="s">
         <v>119</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>120</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>121</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>122</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>123</v>
       </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>124</v>
-      </c>
-      <c r="I13" t="s">
-        <v>125</v>
       </c>
       <c r="J13">
         <v>11953</v>
       </c>
       <c r="K13" t="s">
+        <v>125</v>
+      </c>
+      <c r="L13" t="s">
         <v>126</v>
       </c>
-      <c r="L13" t="s">
+      <c r="M13" t="s">
         <v>127</v>
       </c>
-      <c r="M13" t="s">
+      <c r="N13" t="s">
         <v>128</v>
       </c>
-      <c r="N13" t="s">
+      <c r="O13" t="s">
         <v>129</v>
-      </c>
-      <c r="O13" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.35">
@@ -1878,46 +1891,46 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C14" t="s">
+        <v>130</v>
+      </c>
+      <c r="D14" t="s">
         <v>131</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>132</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>133</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>134</v>
       </c>
-      <c r="G14" t="s">
-        <v>135</v>
-      </c>
       <c r="H14" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I14" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J14">
         <v>90034</v>
       </c>
       <c r="K14" t="s">
+        <v>135</v>
+      </c>
+      <c r="L14" t="s">
         <v>136</v>
       </c>
-      <c r="L14" t="s">
+      <c r="M14" t="s">
         <v>137</v>
       </c>
-      <c r="M14" t="s">
+      <c r="N14" t="s">
         <v>138</v>
       </c>
-      <c r="N14" t="s">
+      <c r="O14" t="s">
         <v>139</v>
-      </c>
-      <c r="O14" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.35">
@@ -1925,46 +1938,46 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C15" t="s">
+        <v>140</v>
+      </c>
+      <c r="D15" t="s">
         <v>141</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>142</v>
       </c>
-      <c r="E15" t="s">
+      <c r="F15" t="s">
         <v>143</v>
       </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>144</v>
       </c>
-      <c r="G15" t="s">
+      <c r="H15" t="s">
         <v>145</v>
       </c>
-      <c r="H15" t="s">
-        <v>146</v>
-      </c>
       <c r="I15" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="J15">
         <v>44023</v>
       </c>
       <c r="K15" t="s">
+        <v>146</v>
+      </c>
+      <c r="L15" t="s">
         <v>147</v>
       </c>
-      <c r="L15" t="s">
+      <c r="M15" t="s">
         <v>148</v>
       </c>
-      <c r="M15" t="s">
+      <c r="N15" t="s">
         <v>149</v>
       </c>
-      <c r="N15" t="s">
+      <c r="O15" t="s">
         <v>150</v>
-      </c>
-      <c r="O15" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.35">
@@ -1972,46 +1985,46 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C16" t="s">
+        <v>151</v>
+      </c>
+      <c r="D16" t="s">
         <v>152</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>153</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>154</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>155</v>
       </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>156</v>
       </c>
-      <c r="H16" t="s">
+      <c r="I16" t="s">
         <v>157</v>
-      </c>
-      <c r="I16" t="s">
-        <v>158</v>
       </c>
       <c r="J16">
         <v>78045</v>
       </c>
       <c r="K16" t="s">
+        <v>158</v>
+      </c>
+      <c r="L16" t="s">
         <v>159</v>
       </c>
-      <c r="L16" t="s">
+      <c r="M16" t="s">
         <v>160</v>
       </c>
-      <c r="M16" t="s">
+      <c r="N16" t="s">
         <v>161</v>
       </c>
-      <c r="N16" t="s">
+      <c r="O16" t="s">
         <v>162</v>
-      </c>
-      <c r="O16" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.35">
@@ -2019,46 +2032,46 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C17" t="s">
+        <v>163</v>
+      </c>
+      <c r="D17" t="s">
         <v>164</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>165</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>166</v>
       </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>167</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>168</v>
       </c>
-      <c r="H17" t="s">
+      <c r="I17" t="s">
         <v>169</v>
-      </c>
-      <c r="I17" t="s">
-        <v>170</v>
       </c>
       <c r="J17">
         <v>85013</v>
       </c>
       <c r="K17" t="s">
+        <v>170</v>
+      </c>
+      <c r="L17" t="s">
         <v>171</v>
       </c>
-      <c r="L17" t="s">
+      <c r="M17" t="s">
         <v>172</v>
       </c>
-      <c r="M17" t="s">
+      <c r="N17" t="s">
         <v>173</v>
       </c>
-      <c r="N17" t="s">
+      <c r="O17" t="s">
         <v>174</v>
-      </c>
-      <c r="O17" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.35">
@@ -2066,46 +2079,46 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C18" t="s">
+        <v>175</v>
+      </c>
+      <c r="D18" t="s">
         <v>176</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>177</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>178</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>179</v>
       </c>
-      <c r="G18" t="s">
+      <c r="H18" t="s">
         <v>180</v>
       </c>
-      <c r="H18" t="s">
+      <c r="I18" t="s">
         <v>181</v>
-      </c>
-      <c r="I18" t="s">
-        <v>182</v>
       </c>
       <c r="J18">
         <v>37110</v>
       </c>
       <c r="K18" t="s">
+        <v>182</v>
+      </c>
+      <c r="L18" t="s">
         <v>183</v>
       </c>
-      <c r="L18" t="s">
+      <c r="M18" t="s">
         <v>184</v>
       </c>
-      <c r="M18" t="s">
+      <c r="N18" t="s">
         <v>185</v>
       </c>
-      <c r="N18" t="s">
+      <c r="O18" t="s">
         <v>186</v>
-      </c>
-      <c r="O18" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.35">
@@ -2113,46 +2126,46 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C19" t="s">
+        <v>187</v>
+      </c>
+      <c r="D19" t="s">
         <v>188</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>189</v>
       </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
         <v>190</v>
       </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
         <v>191</v>
       </c>
-      <c r="G19" t="s">
+      <c r="H19" t="s">
+        <v>191</v>
+      </c>
+      <c r="I19" t="s">
         <v>192</v>
-      </c>
-      <c r="H19" t="s">
-        <v>192</v>
-      </c>
-      <c r="I19" t="s">
-        <v>193</v>
       </c>
       <c r="J19">
         <v>53207</v>
       </c>
       <c r="K19" t="s">
+        <v>193</v>
+      </c>
+      <c r="L19" t="s">
         <v>194</v>
       </c>
-      <c r="L19" t="s">
+      <c r="M19" t="s">
         <v>195</v>
       </c>
-      <c r="M19" t="s">
+      <c r="N19" t="s">
         <v>196</v>
       </c>
-      <c r="N19" t="s">
+      <c r="O19" t="s">
         <v>197</v>
-      </c>
-      <c r="O19" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.35">
@@ -2160,46 +2173,46 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C20" t="s">
+        <v>198</v>
+      </c>
+      <c r="D20" t="s">
         <v>199</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>200</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
         <v>201</v>
       </c>
-      <c r="F20" t="s">
+      <c r="G20" t="s">
         <v>202</v>
       </c>
-      <c r="G20" t="s">
+      <c r="H20" t="s">
         <v>203</v>
       </c>
-      <c r="H20" t="s">
-        <v>204</v>
-      </c>
       <c r="I20" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J20">
         <v>48180</v>
       </c>
       <c r="K20" t="s">
+        <v>204</v>
+      </c>
+      <c r="L20" t="s">
         <v>205</v>
       </c>
-      <c r="L20" t="s">
+      <c r="M20" t="s">
         <v>206</v>
       </c>
-      <c r="M20" t="s">
+      <c r="N20" t="s">
         <v>207</v>
       </c>
-      <c r="N20" t="s">
+      <c r="O20" t="s">
         <v>208</v>
-      </c>
-      <c r="O20" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.35">
@@ -2207,46 +2220,46 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C21" t="s">
+        <v>209</v>
+      </c>
+      <c r="D21" t="s">
         <v>210</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>211</v>
       </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>212</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>213</v>
       </c>
-      <c r="G21" t="s">
+      <c r="H21" t="s">
         <v>214</v>
       </c>
-      <c r="H21" t="s">
-        <v>215</v>
-      </c>
       <c r="I21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J21">
         <v>61109</v>
       </c>
       <c r="K21" t="s">
+        <v>215</v>
+      </c>
+      <c r="L21" t="s">
         <v>216</v>
       </c>
-      <c r="L21" t="s">
+      <c r="M21" t="s">
         <v>217</v>
       </c>
-      <c r="M21" t="s">
+      <c r="N21" t="s">
         <v>218</v>
       </c>
-      <c r="N21" t="s">
+      <c r="O21" t="s">
         <v>219</v>
-      </c>
-      <c r="O21" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.35">
@@ -2254,46 +2267,46 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C22" t="s">
+        <v>220</v>
+      </c>
+      <c r="D22" t="s">
         <v>221</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
         <v>222</v>
       </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
         <v>223</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>224</v>
       </c>
-      <c r="G22" t="s">
+      <c r="H22" t="s">
         <v>225</v>
       </c>
-      <c r="H22" t="s">
-        <v>226</v>
-      </c>
       <c r="I22" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="J22">
         <v>19014</v>
       </c>
       <c r="K22" t="s">
+        <v>226</v>
+      </c>
+      <c r="L22" t="s">
         <v>227</v>
       </c>
-      <c r="L22" t="s">
+      <c r="M22" t="s">
         <v>228</v>
       </c>
-      <c r="M22" t="s">
+      <c r="N22" t="s">
         <v>229</v>
       </c>
-      <c r="N22" t="s">
+      <c r="O22" t="s">
         <v>230</v>
-      </c>
-      <c r="O22" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.35">
@@ -2301,46 +2314,46 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C23" t="s">
+        <v>231</v>
+      </c>
+      <c r="D23" t="s">
         <v>232</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
         <v>233</v>
       </c>
-      <c r="E23" t="s">
+      <c r="F23" t="s">
         <v>234</v>
       </c>
-      <c r="F23" t="s">
-        <v>235</v>
-      </c>
       <c r="G23" t="s">
+        <v>82</v>
+      </c>
+      <c r="H23" t="s">
         <v>83</v>
       </c>
-      <c r="H23" t="s">
+      <c r="I23" t="s">
         <v>84</v>
-      </c>
-      <c r="I23" t="s">
-        <v>85</v>
       </c>
       <c r="J23">
         <v>95111</v>
       </c>
       <c r="K23" t="s">
+        <v>235</v>
+      </c>
+      <c r="L23" t="s">
         <v>236</v>
       </c>
-      <c r="L23" t="s">
+      <c r="M23" t="s">
         <v>237</v>
       </c>
-      <c r="M23" t="s">
+      <c r="N23" t="s">
         <v>238</v>
       </c>
-      <c r="N23" t="s">
+      <c r="O23" t="s">
         <v>239</v>
-      </c>
-      <c r="O23" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.35">
@@ -2348,46 +2361,46 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C24" t="s">
+        <v>240</v>
+      </c>
+      <c r="D24" t="s">
         <v>241</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
         <v>242</v>
       </c>
-      <c r="E24" t="s">
+      <c r="F24" t="s">
         <v>243</v>
       </c>
-      <c r="F24" t="s">
+      <c r="G24" t="s">
         <v>244</v>
       </c>
-      <c r="G24" t="s">
+      <c r="H24" t="s">
         <v>245</v>
       </c>
-      <c r="H24" t="s">
-        <v>246</v>
-      </c>
       <c r="I24" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J24">
         <v>75062</v>
       </c>
       <c r="K24" t="s">
+        <v>246</v>
+      </c>
+      <c r="L24" t="s">
         <v>247</v>
       </c>
-      <c r="L24" t="s">
+      <c r="M24" t="s">
         <v>248</v>
       </c>
-      <c r="M24" t="s">
+      <c r="N24" t="s">
         <v>249</v>
       </c>
-      <c r="N24" t="s">
+      <c r="O24" t="s">
         <v>250</v>
-      </c>
-      <c r="O24" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.35">
@@ -2395,46 +2408,46 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C25" t="s">
+        <v>251</v>
+      </c>
+      <c r="D25" t="s">
         <v>252</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
         <v>253</v>
       </c>
-      <c r="E25" t="s">
+      <c r="F25" t="s">
         <v>254</v>
       </c>
-      <c r="F25" t="s">
+      <c r="G25" t="s">
         <v>255</v>
       </c>
-      <c r="G25" t="s">
-        <v>256</v>
-      </c>
       <c r="H25" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="I25" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J25">
         <v>12204</v>
       </c>
       <c r="K25" t="s">
+        <v>256</v>
+      </c>
+      <c r="L25" t="s">
         <v>257</v>
       </c>
-      <c r="L25" t="s">
+      <c r="M25" t="s">
         <v>258</v>
       </c>
-      <c r="M25" t="s">
+      <c r="N25" t="s">
         <v>259</v>
       </c>
-      <c r="N25" t="s">
+      <c r="O25" t="s">
         <v>260</v>
-      </c>
-      <c r="O25" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.35">
@@ -2442,46 +2455,46 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C26" t="s">
+        <v>261</v>
+      </c>
+      <c r="D26" t="s">
         <v>262</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
         <v>263</v>
       </c>
-      <c r="E26" t="s">
+      <c r="F26" t="s">
         <v>264</v>
       </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
         <v>265</v>
       </c>
-      <c r="G26" t="s">
-        <v>266</v>
-      </c>
       <c r="H26" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="I26" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J26">
         <v>8846</v>
       </c>
       <c r="K26" t="s">
+        <v>266</v>
+      </c>
+      <c r="L26" t="s">
         <v>267</v>
       </c>
-      <c r="L26" t="s">
+      <c r="M26" t="s">
         <v>268</v>
       </c>
-      <c r="M26" t="s">
+      <c r="N26" t="s">
         <v>269</v>
       </c>
-      <c r="N26" t="s">
+      <c r="O26" t="s">
         <v>270</v>
-      </c>
-      <c r="O26" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.35">
@@ -2489,46 +2502,46 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C27" t="s">
+        <v>261</v>
+      </c>
+      <c r="D27" t="s">
         <v>262</v>
       </c>
-      <c r="D27" t="s">
+      <c r="E27" t="s">
         <v>263</v>
       </c>
-      <c r="E27" t="s">
+      <c r="F27" t="s">
         <v>264</v>
       </c>
-      <c r="F27" t="s">
+      <c r="G27" t="s">
         <v>265</v>
       </c>
-      <c r="G27" t="s">
-        <v>266</v>
-      </c>
       <c r="H27" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="I27" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J27">
         <v>8846</v>
       </c>
       <c r="K27" t="s">
+        <v>266</v>
+      </c>
+      <c r="L27" t="s">
         <v>267</v>
       </c>
-      <c r="L27" t="s">
+      <c r="M27" t="s">
         <v>268</v>
       </c>
-      <c r="M27" t="s">
+      <c r="N27" t="s">
         <v>269</v>
       </c>
-      <c r="N27" t="s">
-        <v>270</v>
-      </c>
       <c r="O27" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.35">
@@ -2536,46 +2549,46 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C28" t="s">
+        <v>261</v>
+      </c>
+      <c r="D28" t="s">
         <v>262</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
         <v>263</v>
       </c>
-      <c r="E28" t="s">
-        <v>264</v>
-      </c>
       <c r="F28" t="s">
+        <v>293</v>
+      </c>
+      <c r="G28" t="s">
         <v>265</v>
       </c>
-      <c r="G28" t="s">
-        <v>266</v>
-      </c>
       <c r="H28" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="I28" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J28">
         <v>8846</v>
       </c>
       <c r="K28" t="s">
+        <v>266</v>
+      </c>
+      <c r="L28" t="s">
         <v>267</v>
       </c>
-      <c r="L28" t="s">
+      <c r="M28" t="s">
         <v>268</v>
       </c>
-      <c r="M28" t="s">
+      <c r="N28" t="s">
         <v>269</v>
       </c>
-      <c r="N28" t="s">
-        <v>270</v>
-      </c>
       <c r="O28" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.35">
@@ -2583,46 +2596,46 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C29" t="s">
+        <v>261</v>
+      </c>
+      <c r="D29" t="s">
         <v>262</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" t="s">
         <v>263</v>
       </c>
-      <c r="E29" t="s">
-        <v>264</v>
-      </c>
       <c r="F29" t="s">
+        <v>292</v>
+      </c>
+      <c r="G29" t="s">
         <v>265</v>
       </c>
-      <c r="G29" t="s">
-        <v>266</v>
-      </c>
       <c r="H29" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="I29" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J29">
         <v>8846</v>
       </c>
       <c r="K29" t="s">
+        <v>266</v>
+      </c>
+      <c r="L29" t="s">
         <v>267</v>
       </c>
-      <c r="L29" t="s">
+      <c r="M29" t="s">
         <v>268</v>
       </c>
-      <c r="M29" t="s">
+      <c r="N29" t="s">
         <v>269</v>
       </c>
-      <c r="N29" t="s">
-        <v>270</v>
-      </c>
       <c r="O29" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.35">
@@ -2630,46 +2643,46 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C30" t="s">
+        <v>261</v>
+      </c>
+      <c r="D30" t="s">
         <v>262</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" t="s">
         <v>263</v>
       </c>
-      <c r="E30" t="s">
-        <v>264</v>
-      </c>
       <c r="F30" t="s">
+        <v>291</v>
+      </c>
+      <c r="G30" t="s">
         <v>265</v>
       </c>
-      <c r="G30" t="s">
-        <v>266</v>
-      </c>
       <c r="H30" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="I30" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J30">
         <v>8846</v>
       </c>
       <c r="K30" t="s">
+        <v>266</v>
+      </c>
+      <c r="L30" t="s">
         <v>267</v>
       </c>
-      <c r="L30" t="s">
+      <c r="M30" t="s">
         <v>268</v>
       </c>
-      <c r="M30" t="s">
+      <c r="N30" t="s">
         <v>269</v>
       </c>
-      <c r="N30" t="s">
-        <v>270</v>
-      </c>
       <c r="O30" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
   </sheetData>

</xml_diff>